<commit_message>
Re-verify every defect in real Chrome and correct two reports
All six defects re-tested in Google Chrome with no ad blocking and no suite
fixtures, using user-like interactions (scripts in scripts/repro/, raw results
in docs/bugs/evidence/verification/). All confirmed; two corrected:

- BUG-001: "about:blank" was an automation artifact (Playwright tabs start at
  about:blank). Real impact: "Batal" is a dead button on report links opened in
  a new tab, and sends readers from other sites away. TC-RPT-009 now uses the
  real new-tab path.
- BUG-002: narrowed from intermittent to a deterministic keyboard path (3/3);
  normal scrolling does not trigger it (0/12). TC-RPT-012 is now a real
  known-defect test instead of fixme.

BUG-004/005/006 gained schema, extra boundary values and keyboard evidence.
Final regression: 162 PASS, 7 DEFECT, 0 FLAKY, 0 FAIL, 17 SKIPPED.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -106,7 +106,7 @@
     <t>Logo and login entry visible; at least 3 headline cards; story titles not empty</t>
   </si>
   <si>
-    <t>NOT RUN</t>
+    <t>PASS</t>
   </si>
   <si>
     <t>tests/web/home/home.spec.ts</t>
@@ -585,20 +585,23 @@
     <t>TC-RPT-009</t>
   </si>
   <si>
-    <t>Cancel on a directly opened report link keeps the user on kumparan</t>
-  </si>
-  <si>
-    <t>Users lost on a blank page</t>
-  </si>
-  <si>
-    <t>Report form opened from a shared/bookmarked link (no history)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open /report/story/&lt;slug&gt; directly
+    <t>"Batal" on a report link opened in a new tab takes the reader out of the form</t>
+  </si>
+  <si>
+    <t>Readers stuck on the form (dead Cancel button)</t>
+  </si>
+  <si>
+    <t>Report link opened in a new tab (history.length 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open /report/story/&lt;slug&gt; in a new tab
 2. Click "Batal"</t>
   </si>
   <si>
-    <t>User stays on kumparan (e.g. the story)</t>
+    <t>Reader leaves the form (e.g. back to the story)</t>
+  </si>
+  <si>
+    <t>DEFECT</t>
   </si>
   <si>
     <t>BUG-001</t>
@@ -639,21 +642,24 @@
     <t>TC-RPT-012</t>
   </si>
   <si>
-    <t>Report form keeps its own URL after opening from a story</t>
+    <t>Keyboard user opening the report form keeps the form URL in the address bar</t>
   </si>
   <si>
     <t>Refresh/share leads to a different page than shown</t>
   </si>
   <si>
-    <t>Story read to the end</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Scroll to the end of a story
-2. Open the report form
+    <t>Story open on desktop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Focus "Laporkan tulisan" with the keyboard
+2. Press Enter
 3. Watch the address bar for 4 s</t>
   </si>
   <si>
     <t>URL stays /report/story/&lt;slug&gt;</t>
+  </si>
+  <si>
+    <t>SKIPPED</t>
   </si>
   <si>
     <t>BUG-002</t>
@@ -1302,9 +1308,6 @@
     <t>200; no errors; post matches contract; author id 1</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
     <t>tests/api/graphql/queries.spec.ts</t>
   </si>
   <si>
@@ -1570,9 +1573,6 @@
   </si>
   <si>
     <t>post is null</t>
-  </si>
-  <si>
-    <t>DEFECT</t>
   </si>
   <si>
     <t>BUG-004</t>
@@ -1613,7 +1613,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1635,6 +1635,11 @@
         <fgColor rgb="FFFEE4E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F4F7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1648,7 +1653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1660,6 +1665,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2118,19 +2126,19 @@
       <c r="L2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>28</v>
+      <c r="M2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R2" s="2" t="s">
@@ -2177,19 +2185,19 @@
       <c r="L3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>28</v>
+      <c r="M3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R3" s="2" t="s">
@@ -2236,11 +2244,11 @@
       <c r="L4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>28</v>
+      <c r="M4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>28</v>
@@ -2248,7 +2256,7 @@
       <c r="P4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="Q4" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R4" s="2" t="s">
@@ -2295,19 +2303,19 @@
       <c r="L5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>28</v>
+      <c r="M5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="Q5" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R5" s="2" t="s">
@@ -2354,11 +2362,11 @@
       <c r="L6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>28</v>
+      <c r="M6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>28</v>
@@ -2366,7 +2374,7 @@
       <c r="P6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q6" s="2" t="s">
+      <c r="Q6" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R6" s="2" t="s">
@@ -2413,11 +2421,11 @@
       <c r="L7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>28</v>
+      <c r="M7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>28</v>
@@ -2425,7 +2433,7 @@
       <c r="P7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q7" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R7" s="2" t="s">
@@ -2472,11 +2480,11 @@
       <c r="L8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>28</v>
+      <c r="M8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>28</v>
@@ -2484,7 +2492,7 @@
       <c r="P8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="Q8" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R8" s="2" t="s">
@@ -2531,11 +2539,11 @@
       <c r="L9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="M9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>28</v>
+      <c r="M9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O9" s="2" t="s">
         <v>28</v>
@@ -2543,7 +2551,7 @@
       <c r="P9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="Q9" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R9" s="2" t="s">
@@ -2590,11 +2598,11 @@
       <c r="L10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="M10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>28</v>
+      <c r="M10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>28</v>
@@ -2602,7 +2610,7 @@
       <c r="P10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="Q10" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R10" s="2" t="s">
@@ -2649,11 +2657,11 @@
       <c r="L11" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="M11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>28</v>
+      <c r="M11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>28</v>
@@ -2661,7 +2669,7 @@
       <c r="P11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="Q11" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R11" s="2" t="s">
@@ -2708,19 +2716,19 @@
       <c r="L12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="M12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>28</v>
+      <c r="M12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q12" s="2" t="s">
+      <c r="Q12" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R12" s="2" t="s">
@@ -2767,19 +2775,19 @@
       <c r="L13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="M13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>28</v>
+      <c r="M13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q13" s="2" t="s">
+      <c r="Q13" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R13" s="2" t="s">
@@ -2826,11 +2834,11 @@
       <c r="L14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="M14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>28</v>
+      <c r="M14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>28</v>
@@ -2838,7 +2846,7 @@
       <c r="P14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q14" s="2" t="s">
+      <c r="Q14" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R14" s="2" t="s">
@@ -2885,11 +2893,11 @@
       <c r="L15" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>28</v>
+      <c r="M15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>28</v>
@@ -2897,7 +2905,7 @@
       <c r="P15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q15" s="2" t="s">
+      <c r="Q15" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R15" s="2" t="s">
@@ -2944,11 +2952,11 @@
       <c r="L16" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="M16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>28</v>
+      <c r="M16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>28</v>
@@ -2956,7 +2964,7 @@
       <c r="P16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="Q16" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R16" s="2" t="s">
@@ -3003,11 +3011,11 @@
       <c r="L17" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="M17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>28</v>
+      <c r="M17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O17" s="2" t="s">
         <v>28</v>
@@ -3015,7 +3023,7 @@
       <c r="P17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="Q17" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R17" s="2" t="s">
@@ -3062,19 +3070,19 @@
       <c r="L18" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="M18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>28</v>
+      <c r="M18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q18" s="2" t="s">
+      <c r="Q18" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R18" s="2" t="s">
@@ -3121,11 +3129,11 @@
       <c r="L19" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>28</v>
+      <c r="M19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O19" s="2" t="s">
         <v>28</v>
@@ -3133,7 +3141,7 @@
       <c r="P19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="Q19" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R19" s="2" t="s">
@@ -3180,11 +3188,11 @@
       <c r="L20" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="M20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>28</v>
+      <c r="M20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>28</v>
@@ -3192,7 +3200,7 @@
       <c r="P20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q20" s="2" t="s">
+      <c r="Q20" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R20" s="2" t="s">
@@ -3239,11 +3247,11 @@
       <c r="L21" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>28</v>
+      <c r="M21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>28</v>
@@ -3251,7 +3259,7 @@
       <c r="P21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q21" s="2" t="s">
+      <c r="Q21" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R21" s="2" t="s">
@@ -3298,11 +3306,11 @@
       <c r="L22" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="M22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>28</v>
+      <c r="M22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N22" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>28</v>
@@ -3310,7 +3318,7 @@
       <c r="P22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q22" s="2" t="s">
+      <c r="Q22" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R22" s="2" t="s">
@@ -3357,11 +3365,11 @@
       <c r="L23" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>28</v>
+      <c r="M23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>28</v>
@@ -3369,7 +3377,7 @@
       <c r="P23" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q23" s="2" t="s">
+      <c r="Q23" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R23" s="2" t="s">
@@ -3416,11 +3424,11 @@
       <c r="L24" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="M24" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>28</v>
+      <c r="M24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>28</v>
@@ -3428,7 +3436,7 @@
       <c r="P24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q24" s="2" t="s">
+      <c r="Q24" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R24" s="2" t="s">
@@ -3475,11 +3483,11 @@
       <c r="L25" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="M25" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>28</v>
+      <c r="M25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>28</v>
@@ -3487,7 +3495,7 @@
       <c r="P25" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q25" s="2" t="s">
+      <c r="Q25" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R25" s="2" t="s">
@@ -3534,11 +3542,11 @@
       <c r="L26" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="M26" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>28</v>
+      <c r="M26" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O26" s="2" t="s">
         <v>28</v>
@@ -3546,7 +3554,7 @@
       <c r="P26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q26" s="2" t="s">
+      <c r="Q26" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R26" s="2" t="s">
@@ -3593,11 +3601,11 @@
       <c r="L27" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>28</v>
+      <c r="M27" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O27" s="2" t="s">
         <v>28</v>
@@ -3605,7 +3613,7 @@
       <c r="P27" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q27" s="2" t="s">
+      <c r="Q27" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R27" s="2" t="s">
@@ -3652,11 +3660,11 @@
       <c r="L28" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>28</v>
+      <c r="M28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O28" s="2" t="s">
         <v>28</v>
@@ -3664,7 +3672,7 @@
       <c r="P28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q28" s="2" t="s">
+      <c r="Q28" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R28" s="2" t="s">
@@ -3711,11 +3719,11 @@
       <c r="L29" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="M29" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>28</v>
+      <c r="M29" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N29" s="4" t="s">
+        <v>189</v>
       </c>
       <c r="O29" s="2" t="s">
         <v>28</v>
@@ -3723,11 +3731,11 @@
       <c r="P29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>31</v>
+      <c r="Q29" s="4" t="s">
+        <v>189</v>
       </c>
       <c r="R29" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S29" s="2" t="s">
         <v>144</v>
@@ -3735,13 +3743,13 @@
     </row>
     <row r="30" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>139</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>68</v>
@@ -3756,7 +3764,7 @@
         <v>25</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>148</v>
@@ -3765,16 +3773,16 @@
         <v>28</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="M30" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>28</v>
+      <c r="M30" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N30" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>28</v>
@@ -3782,7 +3790,7 @@
       <c r="P30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q30" s="2" t="s">
+      <c r="Q30" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R30" s="2" t="s">
@@ -3794,13 +3802,13 @@
     </row>
     <row r="31" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>139</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>68</v>
@@ -3815,25 +3823,25 @@
         <v>25</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>148</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>28</v>
+        <v>200</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N31" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>28</v>
@@ -3841,7 +3849,7 @@
       <c r="P31" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q31" s="2" t="s">
+      <c r="Q31" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R31" s="2" t="s">
@@ -3853,13 +3861,13 @@
     </row>
     <row r="32" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>139</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>40</v>
@@ -3868,31 +3876,31 @@
         <v>79</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>25</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>28</v>
+        <v>206</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N32" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>28</v>
@@ -3900,11 +3908,11 @@
       <c r="P32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q32" s="2" t="s">
-        <v>31</v>
+      <c r="Q32" s="4" t="s">
+        <v>189</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="S32" s="2" t="s">
         <v>144</v>
@@ -3912,13 +3920,13 @@
     </row>
     <row r="33" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>22</v>
@@ -3933,7 +3941,7 @@
         <v>25</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>27</v>
@@ -3942,16 +3950,16 @@
         <v>92</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>28</v>
+        <v>214</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N33" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O33" s="2" t="s">
         <v>28</v>
@@ -3959,25 +3967,25 @@
       <c r="P33" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q33" s="2" t="s">
+      <c r="Q33" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R33" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="34" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>22</v>
@@ -3992,7 +4000,7 @@
         <v>25</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>27</v>
@@ -4001,16 +4009,16 @@
         <v>92</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>28</v>
+        <v>220</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N34" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O34" s="2" t="s">
         <v>28</v>
@@ -4018,25 +4026,25 @@
       <c r="P34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q34" s="2" t="s">
+      <c r="Q34" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R34" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="35" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>22</v>
@@ -4051,25 +4059,25 @@
         <v>25</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>92</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>28</v>
+        <v>226</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>28</v>
@@ -4077,25 +4085,25 @@
       <c r="P35" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="2" t="s">
+      <c r="Q35" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R35" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S35" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>22</v>
@@ -4110,25 +4118,25 @@
         <v>25</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>28</v>
+        <v>232</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O36" s="2" t="s">
         <v>28</v>
@@ -4136,25 +4144,25 @@
       <c r="P36" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q36" s="2" t="s">
+      <c r="Q36" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S36" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>40</v>
@@ -4169,7 +4177,7 @@
         <v>25</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>27</v>
@@ -4178,16 +4186,16 @@
         <v>28</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>28</v>
+        <v>237</v>
+      </c>
+      <c r="M37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O37" s="2" t="s">
         <v>28</v>
@@ -4195,25 +4203,25 @@
       <c r="P37" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q37" s="2" t="s">
+      <c r="Q37" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R37" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S37" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>40</v>
@@ -4228,25 +4236,25 @@
         <v>25</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>28</v>
+        <v>242</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O38" s="2" t="s">
         <v>28</v>
@@ -4254,25 +4262,25 @@
       <c r="P38" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q38" s="2" t="s">
+      <c r="Q38" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S38" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="39" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>22</v>
@@ -4287,51 +4295,51 @@
         <v>25</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O39" s="2" t="s">
-        <v>28</v>
+        <v>249</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q39" s="2" t="s">
+      <c r="Q39" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R39" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S39" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>22</v>
@@ -4346,25 +4354,25 @@
         <v>25</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>28</v>
+        <v>256</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>28</v>
@@ -4372,25 +4380,25 @@
       <c r="P40" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q40" s="2" t="s">
+      <c r="Q40" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R40" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="41" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>22</v>
@@ -4405,25 +4413,25 @@
         <v>25</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>28</v>
+        <v>261</v>
+      </c>
+      <c r="M41" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>28</v>
@@ -4431,25 +4439,25 @@
       <c r="P41" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q41" s="2" t="s">
+      <c r="Q41" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R41" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S41" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>55</v>
@@ -4464,25 +4472,25 @@
         <v>25</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>28</v>
+        <v>267</v>
+      </c>
+      <c r="M42" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O42" s="2" t="s">
         <v>28</v>
@@ -4490,25 +4498,25 @@
       <c r="P42" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q42" s="2" t="s">
+      <c r="Q42" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R42" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S42" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="43" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>68</v>
@@ -4523,7 +4531,7 @@
         <v>25</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>27</v>
@@ -4532,16 +4540,16 @@
         <v>28</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N43" s="2" t="s">
-        <v>28</v>
+        <v>272</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O43" s="2" t="s">
         <v>28</v>
@@ -4549,25 +4557,25 @@
       <c r="P43" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q43" s="2" t="s">
+      <c r="Q43" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R43" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S43" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="44" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>68</v>
@@ -4582,25 +4590,25 @@
         <v>25</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N44" s="2" t="s">
-        <v>28</v>
+        <v>278</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N44" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O44" s="2" t="s">
         <v>28</v>
@@ -4608,25 +4616,25 @@
       <c r="P44" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q44" s="2" t="s">
+      <c r="Q44" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R44" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S44" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>68</v>
@@ -4641,25 +4649,25 @@
         <v>25</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="M45" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N45" s="2" t="s">
-        <v>28</v>
+        <v>284</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O45" s="2" t="s">
         <v>28</v>
@@ -4667,25 +4675,25 @@
       <c r="P45" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q45" s="2" t="s">
+      <c r="Q45" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R45" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S45" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>40</v>
@@ -4700,25 +4708,25 @@
         <v>25</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N46" s="2" t="s">
-        <v>28</v>
+        <v>290</v>
+      </c>
+      <c r="M46" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O46" s="2" t="s">
         <v>28</v>
@@ -4726,25 +4734,25 @@
       <c r="P46" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q46" s="2" t="s">
+      <c r="Q46" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R46" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S46" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>40</v>
@@ -4759,25 +4767,25 @@
         <v>25</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N47" s="2" t="s">
-        <v>28</v>
+        <v>296</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O47" s="2" t="s">
         <v>28</v>
@@ -4785,25 +4793,25 @@
       <c r="P47" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q47" s="2" t="s">
+      <c r="Q47" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R47" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S47" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="48" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>40</v>
@@ -4818,25 +4826,25 @@
         <v>25</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="M48" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N48" s="2" t="s">
-        <v>28</v>
+        <v>302</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O48" s="2" t="s">
         <v>28</v>
@@ -4844,25 +4852,25 @@
       <c r="P48" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q48" s="2" t="s">
+      <c r="Q48" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R48" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S48" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>22</v>
@@ -4877,7 +4885,7 @@
         <v>25</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>27</v>
@@ -4886,16 +4894,16 @@
         <v>28</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N49" s="2" t="s">
-        <v>28</v>
+        <v>308</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>28</v>
@@ -4903,25 +4911,25 @@
       <c r="P49" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q49" s="2" t="s">
+      <c r="Q49" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R49" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S49" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="50" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>22</v>
@@ -4936,25 +4944,25 @@
         <v>25</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N50" s="2" t="s">
-        <v>28</v>
+        <v>315</v>
+      </c>
+      <c r="M50" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N50" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>28</v>
@@ -4962,25 +4970,25 @@
       <c r="P50" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q50" s="2" t="s">
+      <c r="Q50" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R50" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S50" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="51" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>22</v>
@@ -4995,25 +5003,25 @@
         <v>25</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N51" s="2" t="s">
-        <v>28</v>
+        <v>321</v>
+      </c>
+      <c r="M51" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N51" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>28</v>
@@ -5021,25 +5029,25 @@
       <c r="P51" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q51" s="2" t="s">
+      <c r="Q51" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R51" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="52" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>22</v>
@@ -5054,25 +5062,25 @@
         <v>25</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N52" s="2" t="s">
-        <v>28</v>
+        <v>327</v>
+      </c>
+      <c r="M52" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>28</v>
@@ -5080,25 +5088,25 @@
       <c r="P52" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q52" s="2" t="s">
+      <c r="Q52" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R52" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="53" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>40</v>
@@ -5113,7 +5121,7 @@
         <v>25</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>27</v>
@@ -5122,16 +5130,16 @@
         <v>28</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N53" s="2" t="s">
-        <v>28</v>
+        <v>332</v>
+      </c>
+      <c r="M53" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N53" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O53" s="2" t="s">
         <v>28</v>
@@ -5139,25 +5147,25 @@
       <c r="P53" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q53" s="2" t="s">
-        <v>31</v>
+      <c r="Q53" s="4" t="s">
+        <v>189</v>
       </c>
       <c r="R53" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="S53" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="54" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>22</v>
@@ -5172,25 +5180,25 @@
         <v>25</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="M54" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N54" s="2" t="s">
-        <v>28</v>
+        <v>327</v>
+      </c>
+      <c r="M54" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N54" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>28</v>
@@ -5198,25 +5206,25 @@
       <c r="P54" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q54" s="2" t="s">
+      <c r="Q54" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R54" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S54" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="55" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>22</v>
@@ -5228,10 +5236,10 @@
         <v>12</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>27</v>
@@ -5240,16 +5248,16 @@
         <v>28</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N55" s="2" t="s">
-        <v>28</v>
+        <v>344</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N55" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O55" s="2" t="s">
         <v>28</v>
@@ -5257,25 +5265,25 @@
       <c r="P55" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q55" s="2" t="s">
+      <c r="Q55" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R55" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S55" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="56" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>55</v>
@@ -5287,10 +5295,10 @@
         <v>12</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>27</v>
@@ -5299,16 +5307,16 @@
         <v>28</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>28</v>
+        <v>349</v>
+      </c>
+      <c r="M56" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N56" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>28</v>
@@ -5316,25 +5324,25 @@
       <c r="P56" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q56" s="2" t="s">
+      <c r="Q56" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R56" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S56" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="57" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>68</v>
@@ -5346,10 +5354,10 @@
         <v>12</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>27</v>
@@ -5358,16 +5366,16 @@
         <v>28</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M57" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N57" s="2" t="s">
-        <v>28</v>
+        <v>354</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N57" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>28</v>
@@ -5375,25 +5383,25 @@
       <c r="P57" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q57" s="2" t="s">
+      <c r="Q57" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R57" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S57" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="58" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>40</v>
@@ -5405,10 +5413,10 @@
         <v>12</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>27</v>
@@ -5417,16 +5425,16 @@
         <v>28</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>28</v>
+        <v>359</v>
+      </c>
+      <c r="M58" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N58" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>28</v>
@@ -5434,25 +5442,25 @@
       <c r="P58" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q58" s="2" t="s">
+      <c r="Q58" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R58" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S58" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="59" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>22</v>
@@ -5464,10 +5472,10 @@
         <v>12</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>27</v>
@@ -5476,16 +5484,16 @@
         <v>28</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="M59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N59" s="2" t="s">
-        <v>28</v>
+        <v>363</v>
+      </c>
+      <c r="M59" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N59" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O59" s="2" t="s">
         <v>28</v>
@@ -5493,25 +5501,25 @@
       <c r="P59" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q59" s="2" t="s">
+      <c r="Q59" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R59" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S59" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="60" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>40</v>
@@ -5523,10 +5531,10 @@
         <v>12</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>27</v>
@@ -5535,16 +5543,16 @@
         <v>28</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>28</v>
+        <v>369</v>
+      </c>
+      <c r="M60" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N60" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O60" s="2" t="s">
         <v>28</v>
@@ -5552,25 +5560,25 @@
       <c r="P60" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q60" s="2" t="s">
+      <c r="Q60" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R60" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="61" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>22</v>
@@ -5582,10 +5590,10 @@
         <v>12</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>27</v>
@@ -5594,16 +5602,16 @@
         <v>28</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>28</v>
+        <v>374</v>
+      </c>
+      <c r="M61" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N61" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O61" s="2" t="s">
         <v>28</v>
@@ -5611,25 +5619,25 @@
       <c r="P61" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q61" s="2" t="s">
+      <c r="Q61" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R61" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S61" s="2" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="62" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>40</v>
@@ -5641,10 +5649,10 @@
         <v>12</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>27</v>
@@ -5653,16 +5661,16 @@
         <v>28</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="M62" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N62" s="2" t="s">
-        <v>28</v>
+        <v>380</v>
+      </c>
+      <c r="M62" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N62" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O62" s="2" t="s">
         <v>28</v>
@@ -5670,25 +5678,25 @@
       <c r="P62" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q62" s="2" t="s">
+      <c r="Q62" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R62" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S62" s="2" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="63" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>55</v>
@@ -5700,28 +5708,28 @@
         <v>12</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="M63" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N63" s="2" t="s">
-        <v>28</v>
+        <v>385</v>
+      </c>
+      <c r="M63" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N63" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="O63" s="2" t="s">
         <v>28</v>
@@ -5729,25 +5737,25 @@
       <c r="P63" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q63" s="2" t="s">
-        <v>31</v>
+      <c r="Q63" s="4" t="s">
+        <v>189</v>
       </c>
       <c r="R63" s="2" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="S63" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="64" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>22</v>
@@ -5759,28 +5767,28 @@
         <v>13</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="M64" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N64" s="2" t="s">
-        <v>28</v>
+        <v>391</v>
+      </c>
+      <c r="M64" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N64" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O64" s="2" t="s">
         <v>28</v>
@@ -5788,25 +5796,25 @@
       <c r="P64" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q64" s="2" t="s">
+      <c r="Q64" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R64" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S64" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="65" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>22</v>
@@ -5818,28 +5826,28 @@
         <v>13</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="M65" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N65" s="2" t="s">
-        <v>28</v>
+        <v>396</v>
+      </c>
+      <c r="M65" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N65" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O65" s="2" t="s">
         <v>28</v>
@@ -5847,25 +5855,25 @@
       <c r="P65" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q65" s="2" t="s">
+      <c r="Q65" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R65" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S65" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="66" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>22</v>
@@ -5877,28 +5885,28 @@
         <v>13</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J66" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="M66" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N66" s="2" t="s">
-        <v>28</v>
+        <v>401</v>
+      </c>
+      <c r="M66" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N66" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O66" s="2" t="s">
         <v>28</v>
@@ -5906,25 +5914,25 @@
       <c r="P66" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q66" s="2" t="s">
+      <c r="Q66" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R66" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S66" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="67" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>22</v>
@@ -5936,28 +5944,28 @@
         <v>13</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="L67" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="M67" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N67" s="2" t="s">
-        <v>28</v>
+        <v>406</v>
+      </c>
+      <c r="M67" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="N67" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="O67" s="2" t="s">
         <v>28</v>
@@ -5965,25 +5973,25 @@
       <c r="P67" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q67" s="2" t="s">
+      <c r="Q67" s="3" t="s">
         <v>31</v>
       </c>
       <c r="R67" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S67" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="68" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>22</v>
@@ -5998,19 +6006,19 @@
         <v>25</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="M68" s="2" t="s">
         <v>28</v>
@@ -6022,27 +6030,27 @@
         <v>28</v>
       </c>
       <c r="P68" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q68" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R68" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S68" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="69" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>22</v>
@@ -6057,19 +6065,19 @@
         <v>25</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M69" s="2" t="s">
         <v>28</v>
@@ -6081,27 +6089,27 @@
         <v>28</v>
       </c>
       <c r="P69" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q69" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R69" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S69" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="70" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>22</v>
@@ -6116,19 +6124,19 @@
         <v>25</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="M70" s="2" t="s">
         <v>28</v>
@@ -6140,27 +6148,27 @@
         <v>28</v>
       </c>
       <c r="P70" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q70" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R70" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S70" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="71" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>22</v>
@@ -6175,19 +6183,19 @@
         <v>25</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="M71" s="2" t="s">
         <v>28</v>
@@ -6199,27 +6207,27 @@
         <v>28</v>
       </c>
       <c r="P71" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q71" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R71" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S71" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="72" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>22</v>
@@ -6234,19 +6242,19 @@
         <v>25</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="M72" s="2" t="s">
         <v>28</v>
@@ -6258,27 +6266,27 @@
         <v>28</v>
       </c>
       <c r="P72" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q72" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R72" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S72" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="73" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>22</v>
@@ -6293,19 +6301,19 @@
         <v>25</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="M73" s="2" t="s">
         <v>28</v>
@@ -6317,27 +6325,27 @@
         <v>28</v>
       </c>
       <c r="P73" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q73" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R73" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S73" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="74" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>68</v>
@@ -6352,19 +6360,19 @@
         <v>25</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="M74" s="2" t="s">
         <v>28</v>
@@ -6376,27 +6384,27 @@
         <v>28</v>
       </c>
       <c r="P74" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q74" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R74" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S74" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="75" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>22</v>
@@ -6411,19 +6419,19 @@
         <v>25</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J75" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L75" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="M75" s="2" t="s">
         <v>28</v>
@@ -6435,27 +6443,27 @@
         <v>28</v>
       </c>
       <c r="P75" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q75" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R75" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S75" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="76" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>22</v>
@@ -6470,19 +6478,19 @@
         <v>25</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="I76" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="L76" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="M76" s="2" t="s">
         <v>28</v>
@@ -6494,27 +6502,27 @@
         <v>28</v>
       </c>
       <c r="P76" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q76" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R76" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S76" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="77" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>22</v>
@@ -6529,19 +6537,19 @@
         <v>25</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J77" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K77" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="L77" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M77" s="2" t="s">
         <v>28</v>
@@ -6553,27 +6561,27 @@
         <v>28</v>
       </c>
       <c r="P77" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q77" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R77" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S77" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="78" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>55</v>
@@ -6588,19 +6596,19 @@
         <v>25</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="I78" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J78" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L78" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="M78" s="2" t="s">
         <v>28</v>
@@ -6612,27 +6620,27 @@
         <v>28</v>
       </c>
       <c r="P78" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q78" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R78" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S78" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="79" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>55</v>
@@ -6647,19 +6655,19 @@
         <v>25</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J79" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="L79" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="M79" s="2" t="s">
         <v>28</v>
@@ -6671,27 +6679,27 @@
         <v>28</v>
       </c>
       <c r="P79" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q79" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R79" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S79" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="80" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>55</v>
@@ -6706,19 +6714,19 @@
         <v>25</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J80" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="M80" s="2" t="s">
         <v>28</v>
@@ -6730,27 +6738,27 @@
         <v>28</v>
       </c>
       <c r="P80" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q80" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R80" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S80" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="81" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>55</v>
@@ -6765,19 +6773,19 @@
         <v>25</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J81" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K81" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="L81" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="M81" s="2" t="s">
         <v>28</v>
@@ -6789,27 +6797,27 @@
         <v>28</v>
       </c>
       <c r="P81" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q81" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R81" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S81" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="82" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>55</v>
@@ -6824,19 +6832,19 @@
         <v>25</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J82" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="L82" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="M82" s="2" t="s">
         <v>28</v>
@@ -6848,27 +6856,27 @@
         <v>28</v>
       </c>
       <c r="P82" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q82" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R82" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S82" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="83" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>40</v>
@@ -6883,19 +6891,19 @@
         <v>25</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="I83" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J83" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K83" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="L83" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="M83" s="2" t="s">
         <v>28</v>
@@ -6907,27 +6915,27 @@
         <v>28</v>
       </c>
       <c r="P83" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q83" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R83" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S83" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="84" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>55</v>
@@ -6942,19 +6950,19 @@
         <v>25</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="I84" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J84" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K84" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="L84" s="2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M84" s="2" t="s">
         <v>28</v>
@@ -6966,27 +6974,27 @@
         <v>28</v>
       </c>
       <c r="P84" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="Q84" s="3" t="s">
-        <v>413</v>
+        <v>31</v>
       </c>
       <c r="R84" s="2" t="s">
         <v>28</v>
       </c>
       <c r="S84" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="85" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>68</v>
@@ -7001,19 +7009,19 @@
         <v>25</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="I85" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J85" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="L85" s="2" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="M85" s="2" t="s">
         <v>28</v>
@@ -7025,16 +7033,16 @@
         <v>28</v>
       </c>
       <c r="P85" s="4" t="s">
-        <v>503</v>
+        <v>189</v>
       </c>
       <c r="Q85" s="4" t="s">
-        <v>503</v>
+        <v>189</v>
       </c>
       <c r="R85" s="2" t="s">
         <v>504</v>
       </c>
       <c r="S85" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="86" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7042,7 +7050,7 @@
         <v>505</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>506</v>
@@ -7063,7 +7071,7 @@
         <v>507</v>
       </c>
       <c r="I86" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J86" s="2" t="s">
         <v>28</v>
@@ -7084,16 +7092,16 @@
         <v>28</v>
       </c>
       <c r="P86" s="4" t="s">
-        <v>503</v>
+        <v>189</v>
       </c>
       <c r="Q86" s="4" t="s">
-        <v>503</v>
+        <v>189</v>
       </c>
       <c r="R86" s="2" t="s">
         <v>510</v>
       </c>
       <c r="S86" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schedule platform-specific tests only where they apply (no skips)
Desktop-only and mobile-only tests carry @desktop-only / @mobile-only tags and
are excluded per project with grepInvert; agent spec folders are scoped with
testIgnore. Full regression: 169 executions, 162 PASS, 7 DEFECT, 0 FLAKY,
0 FAIL, 0 SKIPPED.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1634" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1634" uniqueCount="510">
   <si>
     <t>ID</t>
   </si>
@@ -657,9 +657,6 @@
   </si>
   <si>
     <t>URL stays /report/story/&lt;slug&gt;</t>
-  </si>
-  <si>
-    <t>SKIPPED</t>
   </si>
   <si>
     <t>BUG-002</t>
@@ -1613,7 +1610,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1635,11 +1632,6 @@
         <fgColor rgb="FFFEE4E2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F4F7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1653,7 +1645,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1665,9 +1657,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3899,8 +3888,8 @@
       <c r="M32" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="N32" s="5" t="s">
-        <v>207</v>
+      <c r="N32" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>28</v>
@@ -3912,7 +3901,7 @@
         <v>189</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S32" s="2" t="s">
         <v>144</v>
@@ -3920,13 +3909,13 @@
     </row>
     <row r="33" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>22</v>
@@ -3941,7 +3930,7 @@
         <v>25</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>27</v>
@@ -3950,42 +3939,42 @@
         <v>92</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="M33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S33" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="M33" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N33" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P33" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q33" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S33" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="34" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>22</v>
@@ -4000,7 +3989,7 @@
         <v>25</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>27</v>
@@ -4009,11 +3998,11 @@
         <v>92</v>
       </c>
       <c r="K34" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="L34" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="L34" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="M34" s="3" t="s">
         <v>31</v>
       </c>
@@ -4033,18 +4022,18 @@
         <v>28</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>22</v>
@@ -4059,20 +4048,20 @@
         <v>25</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>224</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>92</v>
       </c>
       <c r="K35" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="L35" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="L35" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="M35" s="3" t="s">
         <v>31</v>
       </c>
@@ -4092,18 +4081,18 @@
         <v>28</v>
       </c>
       <c r="S35" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="36" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>228</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>22</v>
@@ -4118,20 +4107,20 @@
         <v>25</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="J36" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K36" s="2" t="s">
+      <c r="L36" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="L36" s="2" t="s">
-        <v>232</v>
-      </c>
       <c r="M36" s="3" t="s">
         <v>31</v>
       </c>
@@ -4151,18 +4140,18 @@
         <v>28</v>
       </c>
       <c r="S36" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>234</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>40</v>
@@ -4177,7 +4166,7 @@
         <v>25</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>27</v>
@@ -4186,11 +4175,11 @@
         <v>28</v>
       </c>
       <c r="K37" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="L37" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="M37" s="3" t="s">
         <v>31</v>
       </c>
@@ -4210,18 +4199,18 @@
         <v>28</v>
       </c>
       <c r="S37" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>239</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>40</v>
@@ -4236,20 +4225,20 @@
         <v>25</v>
       </c>
       <c r="H38" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K38" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="I38" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K38" s="2" t="s">
+      <c r="L38" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="L38" s="2" t="s">
-        <v>242</v>
-      </c>
       <c r="M38" s="3" t="s">
         <v>31</v>
       </c>
@@ -4269,18 +4258,18 @@
         <v>28</v>
       </c>
       <c r="S38" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="39" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>245</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>22</v>
@@ -4295,51 +4284,51 @@
         <v>25</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="K39" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="L39" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="M39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S39" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="M39" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N39" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O39" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P39" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q39" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R39" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>252</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>22</v>
@@ -4354,20 +4343,20 @@
         <v>25</v>
       </c>
       <c r="H40" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="J40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K40" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="J40" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K40" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="L40" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="M40" s="3" t="s">
         <v>31</v>
       </c>
@@ -4387,18 +4376,18 @@
         <v>28</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="41" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>22</v>
@@ -4413,20 +4402,20 @@
         <v>25</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K41" s="2" t="s">
+      <c r="L41" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>261</v>
-      </c>
       <c r="M41" s="3" t="s">
         <v>31</v>
       </c>
@@ -4446,18 +4435,18 @@
         <v>28</v>
       </c>
       <c r="S41" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="42" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>263</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>55</v>
@@ -4472,20 +4461,20 @@
         <v>25</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J42" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="L42" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="L42" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="M42" s="3" t="s">
         <v>31</v>
       </c>
@@ -4505,18 +4494,18 @@
         <v>28</v>
       </c>
       <c r="S42" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="43" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>269</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>68</v>
@@ -4531,7 +4520,7 @@
         <v>25</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>27</v>
@@ -4540,11 +4529,11 @@
         <v>28</v>
       </c>
       <c r="K43" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="L43" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="L43" s="2" t="s">
-        <v>272</v>
-      </c>
       <c r="M43" s="3" t="s">
         <v>31</v>
       </c>
@@ -4564,18 +4553,18 @@
         <v>28</v>
       </c>
       <c r="S43" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>273</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>274</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>68</v>
@@ -4590,20 +4579,20 @@
         <v>25</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J44" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="K44" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="L44" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="L44" s="2" t="s">
-        <v>278</v>
-      </c>
       <c r="M44" s="3" t="s">
         <v>31</v>
       </c>
@@ -4623,18 +4612,18 @@
         <v>28</v>
       </c>
       <c r="S44" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="45" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>68</v>
@@ -4649,20 +4638,20 @@
         <v>25</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J45" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="K45" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="L45" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="L45" s="2" t="s">
-        <v>284</v>
-      </c>
       <c r="M45" s="3" t="s">
         <v>31</v>
       </c>
@@ -4682,18 +4671,18 @@
         <v>28</v>
       </c>
       <c r="S45" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>285</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>40</v>
@@ -4708,20 +4697,20 @@
         <v>25</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J46" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="K46" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="K46" s="2" t="s">
+      <c r="L46" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="L46" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="M46" s="3" t="s">
         <v>31</v>
       </c>
@@ -4741,18 +4730,18 @@
         <v>28</v>
       </c>
       <c r="S46" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>40</v>
@@ -4767,20 +4756,20 @@
         <v>25</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J47" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K47" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="L47" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="L47" s="2" t="s">
-        <v>296</v>
-      </c>
       <c r="M47" s="3" t="s">
         <v>31</v>
       </c>
@@ -4800,18 +4789,18 @@
         <v>28</v>
       </c>
       <c r="S47" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="48" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>297</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>298</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>40</v>
@@ -4826,20 +4815,20 @@
         <v>25</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J48" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="K48" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="L48" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="L48" s="2" t="s">
-        <v>302</v>
-      </c>
       <c r="M48" s="3" t="s">
         <v>31</v>
       </c>
@@ -4859,18 +4848,18 @@
         <v>28</v>
       </c>
       <c r="S48" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>304</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>305</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>22</v>
@@ -4885,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>27</v>
@@ -4894,42 +4883,42 @@
         <v>28</v>
       </c>
       <c r="K49" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="L49" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="M49" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S49" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="M49" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N49" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q49" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S49" s="2" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="50" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>22</v>
@@ -4944,22 +4933,22 @@
         <v>25</v>
       </c>
       <c r="H50" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="I50" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="J50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K50" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="J50" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K50" s="2" t="s">
+      <c r="L50" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="L50" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="M50" s="5" t="s">
-        <v>207</v>
+      <c r="M50" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="N50" s="3" t="s">
         <v>31</v>
@@ -4977,18 +4966,18 @@
         <v>28</v>
       </c>
       <c r="S50" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="51" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>317</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>22</v>
@@ -5003,20 +4992,20 @@
         <v>25</v>
       </c>
       <c r="H51" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="I51" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="J51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K51" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="J51" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K51" s="2" t="s">
+      <c r="L51" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="L51" s="2" t="s">
-        <v>321</v>
-      </c>
       <c r="M51" s="3" t="s">
         <v>31</v>
       </c>
@@ -5036,18 +5025,18 @@
         <v>28</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="52" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>322</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>323</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>22</v>
@@ -5062,25 +5051,25 @@
         <v>25</v>
       </c>
       <c r="H52" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="I52" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="I52" s="2" t="s">
+      <c r="J52" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K52" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="J52" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K52" s="2" t="s">
+      <c r="L52" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="L52" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="M52" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N52" s="5" t="s">
-        <v>207</v>
+      <c r="N52" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>28</v>
@@ -5095,18 +5084,18 @@
         <v>28</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="53" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>328</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>329</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>40</v>
@@ -5121,7 +5110,7 @@
         <v>25</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>27</v>
@@ -5130,10 +5119,10 @@
         <v>28</v>
       </c>
       <c r="K53" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="L53" s="2" t="s">
         <v>331</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>332</v>
       </c>
       <c r="M53" s="4" t="s">
         <v>189</v>
@@ -5151,21 +5140,21 @@
         <v>189</v>
       </c>
       <c r="R53" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="S53" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="54" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>335</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>22</v>
@@ -5180,22 +5169,22 @@
         <v>25</v>
       </c>
       <c r="H54" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K54" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="I54" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>337</v>
-      </c>
       <c r="L54" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="M54" s="5" t="s">
-        <v>207</v>
+        <v>326</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="N54" s="3" t="s">
         <v>31</v>
@@ -5213,18 +5202,18 @@
         <v>28</v>
       </c>
       <c r="S54" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="55" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>340</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>22</v>
@@ -5236,10 +5225,10 @@
         <v>12</v>
       </c>
       <c r="G55" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="H55" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>342</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>27</v>
@@ -5248,42 +5237,42 @@
         <v>28</v>
       </c>
       <c r="K55" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="L55" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="L55" s="2" t="s">
+      <c r="M55" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q55" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S55" s="2" t="s">
         <v>344</v>
-      </c>
-      <c r="M55" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N55" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="O55" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P55" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q55" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R55" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S55" s="2" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="56" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>346</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>347</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>55</v>
@@ -5295,10 +5284,10 @@
         <v>12</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>27</v>
@@ -5307,16 +5296,16 @@
         <v>28</v>
       </c>
       <c r="K56" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="L56" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="L56" s="2" t="s">
-        <v>349</v>
-      </c>
       <c r="M56" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N56" s="5" t="s">
-        <v>207</v>
+      <c r="N56" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>28</v>
@@ -5331,18 +5320,18 @@
         <v>28</v>
       </c>
       <c r="S56" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="57" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>350</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>351</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>68</v>
@@ -5354,10 +5343,10 @@
         <v>12</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>27</v>
@@ -5366,16 +5355,16 @@
         <v>28</v>
       </c>
       <c r="K57" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="L57" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="L57" s="2" t="s">
-        <v>354</v>
-      </c>
       <c r="M57" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N57" s="5" t="s">
-        <v>207</v>
+      <c r="N57" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>28</v>
@@ -5390,18 +5379,18 @@
         <v>28</v>
       </c>
       <c r="S57" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="58" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>355</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>356</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>40</v>
@@ -5413,10 +5402,10 @@
         <v>12</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>27</v>
@@ -5425,16 +5414,16 @@
         <v>28</v>
       </c>
       <c r="K58" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="L58" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="L58" s="2" t="s">
-        <v>359</v>
-      </c>
       <c r="M58" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N58" s="5" t="s">
-        <v>207</v>
+      <c r="N58" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>28</v>
@@ -5449,18 +5438,18 @@
         <v>28</v>
       </c>
       <c r="S58" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="59" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>360</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>361</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>22</v>
@@ -5472,10 +5461,10 @@
         <v>12</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>27</v>
@@ -5484,42 +5473,42 @@
         <v>28</v>
       </c>
       <c r="K59" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="L59" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="L59" s="2" t="s">
+      <c r="M59" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q59" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S59" s="2" t="s">
         <v>363</v>
-      </c>
-      <c r="M59" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N59" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="O59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q59" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S59" s="2" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="60" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>365</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>366</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>40</v>
@@ -5531,10 +5520,10 @@
         <v>12</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>27</v>
@@ -5543,16 +5532,16 @@
         <v>28</v>
       </c>
       <c r="K60" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="L60" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="L60" s="2" t="s">
-        <v>369</v>
-      </c>
       <c r="M60" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N60" s="5" t="s">
-        <v>207</v>
+      <c r="N60" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O60" s="2" t="s">
         <v>28</v>
@@ -5567,18 +5556,18 @@
         <v>28</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="61" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>370</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>371</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>22</v>
@@ -5590,10 +5579,10 @@
         <v>12</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>27</v>
@@ -5602,42 +5591,42 @@
         <v>28</v>
       </c>
       <c r="K61" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="L61" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="L61" s="2" t="s">
+      <c r="M61" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q61" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S61" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="M61" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N61" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="O61" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P61" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q61" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R61" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S61" s="2" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="62" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>377</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>40</v>
@@ -5649,10 +5638,10 @@
         <v>12</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>27</v>
@@ -5661,16 +5650,16 @@
         <v>28</v>
       </c>
       <c r="K62" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="L62" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="L62" s="2" t="s">
-        <v>380</v>
-      </c>
       <c r="M62" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N62" s="5" t="s">
-        <v>207</v>
+      <c r="N62" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O62" s="2" t="s">
         <v>28</v>
@@ -5685,18 +5674,18 @@
         <v>28</v>
       </c>
       <c r="S62" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="63" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>382</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>55</v>
@@ -5708,28 +5697,28 @@
         <v>12</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H63" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K63" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="I63" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="J63" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K63" s="2" t="s">
+      <c r="L63" s="2" t="s">
         <v>384</v>
-      </c>
-      <c r="L63" s="2" t="s">
-        <v>385</v>
       </c>
       <c r="M63" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="N63" s="5" t="s">
-        <v>207</v>
+      <c r="N63" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="O63" s="2" t="s">
         <v>28</v>
@@ -5741,21 +5730,21 @@
         <v>189</v>
       </c>
       <c r="R63" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="S63" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="64" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>387</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>388</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>22</v>
@@ -5767,54 +5756,54 @@
         <v>13</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H64" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K64" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="J64" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K64" s="2" t="s">
+      <c r="L64" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="L64" s="2" t="s">
+      <c r="M64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N64" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q64" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S64" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="M64" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="N64" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="O64" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P64" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q64" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R64" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S64" s="2" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="65" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>393</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>394</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>22</v>
@@ -5826,25 +5815,25 @@
         <v>13</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K65" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="L65" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="L65" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="M65" s="5" t="s">
-        <v>207</v>
+      <c r="M65" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="N65" s="3" t="s">
         <v>31</v>
@@ -5862,18 +5851,18 @@
         <v>28</v>
       </c>
       <c r="S65" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="66" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>397</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>398</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>22</v>
@@ -5885,25 +5874,25 @@
         <v>13</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H66" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K66" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="I66" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K66" s="2" t="s">
+      <c r="L66" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="L66" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="M66" s="5" t="s">
-        <v>207</v>
+      <c r="M66" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="N66" s="3" t="s">
         <v>31</v>
@@ -5921,18 +5910,18 @@
         <v>28</v>
       </c>
       <c r="S66" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="67" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>402</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>403</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>22</v>
@@ -5944,25 +5933,25 @@
         <v>13</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H67" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K67" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="I67" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K67" s="2" t="s">
+      <c r="L67" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="M67" s="5" t="s">
-        <v>207</v>
+      <c r="M67" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="N67" s="3" t="s">
         <v>31</v>
@@ -5980,18 +5969,18 @@
         <v>28</v>
       </c>
       <c r="S67" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="68" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>408</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>409</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>22</v>
@@ -6006,51 +5995,51 @@
         <v>25</v>
       </c>
       <c r="H68" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="I68" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="I68" s="2" t="s">
+      <c r="J68" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="J68" s="2" t="s">
+      <c r="K68" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="K68" s="2" t="s">
+      <c r="L68" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="L68" s="2" t="s">
+      <c r="M68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P68" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q68" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S68" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="M68" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N68" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O68" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P68" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q68" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R68" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S68" s="2" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="69" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>416</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>417</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>22</v>
@@ -6065,20 +6054,20 @@
         <v>25</v>
       </c>
       <c r="H69" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J69" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="I69" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J69" s="2" t="s">
+      <c r="K69" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="K69" s="2" t="s">
+      <c r="L69" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="L69" s="2" t="s">
-        <v>421</v>
-      </c>
       <c r="M69" s="2" t="s">
         <v>28</v>
       </c>
@@ -6098,18 +6087,18 @@
         <v>28</v>
       </c>
       <c r="S69" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="70" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>422</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>423</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>22</v>
@@ -6124,20 +6113,20 @@
         <v>25</v>
       </c>
       <c r="H70" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K70" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="I70" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K70" s="2" t="s">
+      <c r="L70" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="L70" s="2" t="s">
-        <v>426</v>
-      </c>
       <c r="M70" s="2" t="s">
         <v>28</v>
       </c>
@@ -6157,18 +6146,18 @@
         <v>28</v>
       </c>
       <c r="S70" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="71" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>428</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>22</v>
@@ -6183,20 +6172,20 @@
         <v>25</v>
       </c>
       <c r="H71" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K71" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="I71" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J71" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K71" s="2" t="s">
+      <c r="L71" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="L71" s="2" t="s">
-        <v>431</v>
-      </c>
       <c r="M71" s="2" t="s">
         <v>28</v>
       </c>
@@ -6216,18 +6205,18 @@
         <v>28</v>
       </c>
       <c r="S71" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="72" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>433</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>22</v>
@@ -6242,20 +6231,20 @@
         <v>25</v>
       </c>
       <c r="H72" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J72" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="I72" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J72" s="2" t="s">
+      <c r="K72" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="K72" s="2" t="s">
+      <c r="L72" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="L72" s="2" t="s">
-        <v>437</v>
-      </c>
       <c r="M72" s="2" t="s">
         <v>28</v>
       </c>
@@ -6275,18 +6264,18 @@
         <v>28</v>
       </c>
       <c r="S72" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="73" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>438</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>22</v>
@@ -6301,20 +6290,20 @@
         <v>25</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>28</v>
       </c>
       <c r="K73" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="L73" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="L73" s="2" t="s">
-        <v>441</v>
-      </c>
       <c r="M73" s="2" t="s">
         <v>28</v>
       </c>
@@ -6334,18 +6323,18 @@
         <v>28</v>
       </c>
       <c r="S73" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="74" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>442</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>443</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>68</v>
@@ -6360,20 +6349,20 @@
         <v>25</v>
       </c>
       <c r="H74" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K74" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="I74" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J74" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K74" s="2" t="s">
+      <c r="L74" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="L74" s="2" t="s">
-        <v>446</v>
-      </c>
       <c r="M74" s="2" t="s">
         <v>28</v>
       </c>
@@ -6393,18 +6382,18 @@
         <v>28</v>
       </c>
       <c r="S74" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="75" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>22</v>
@@ -6419,51 +6408,51 @@
         <v>25</v>
       </c>
       <c r="H75" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K75" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="I75" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K75" s="2" t="s">
+      <c r="L75" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="L75" s="2" t="s">
+      <c r="M75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P75" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q75" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S75" s="2" t="s">
         <v>451</v>
-      </c>
-      <c r="M75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P75" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q75" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S75" s="2" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="76" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>22</v>
@@ -6478,20 +6467,20 @@
         <v>25</v>
       </c>
       <c r="H76" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K76" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="I76" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J76" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K76" s="2" t="s">
+      <c r="L76" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="L76" s="2" t="s">
-        <v>457</v>
-      </c>
       <c r="M76" s="2" t="s">
         <v>28</v>
       </c>
@@ -6511,18 +6500,18 @@
         <v>28</v>
       </c>
       <c r="S76" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="77" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>458</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>459</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>22</v>
@@ -6537,20 +6526,20 @@
         <v>25</v>
       </c>
       <c r="H77" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K77" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="I77" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J77" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K77" s="2" t="s">
+      <c r="L77" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="L77" s="2" t="s">
-        <v>462</v>
-      </c>
       <c r="M77" s="2" t="s">
         <v>28</v>
       </c>
@@ -6570,18 +6559,18 @@
         <v>28</v>
       </c>
       <c r="S77" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="78" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>463</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>464</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>55</v>
@@ -6596,20 +6585,20 @@
         <v>25</v>
       </c>
       <c r="H78" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K78" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="I78" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J78" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K78" s="2" t="s">
+      <c r="L78" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="L78" s="2" t="s">
-        <v>467</v>
-      </c>
       <c r="M78" s="2" t="s">
         <v>28</v>
       </c>
@@ -6629,18 +6618,18 @@
         <v>28</v>
       </c>
       <c r="S78" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="79" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>468</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>469</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>55</v>
@@ -6655,51 +6644,51 @@
         <v>25</v>
       </c>
       <c r="H79" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K79" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="I79" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K79" s="2" t="s">
+      <c r="L79" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="L79" s="2" t="s">
+      <c r="M79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P79" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q79" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S79" s="2" t="s">
         <v>472</v>
-      </c>
-      <c r="M79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P79" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q79" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S79" s="2" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="80" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>474</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>475</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>55</v>
@@ -6714,20 +6703,20 @@
         <v>25</v>
       </c>
       <c r="H80" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K80" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="I80" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J80" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K80" s="2" t="s">
+      <c r="L80" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="L80" s="2" t="s">
-        <v>478</v>
-      </c>
       <c r="M80" s="2" t="s">
         <v>28</v>
       </c>
@@ -6747,18 +6736,18 @@
         <v>28</v>
       </c>
       <c r="S80" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="81" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>479</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>480</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>55</v>
@@ -6773,20 +6762,20 @@
         <v>25</v>
       </c>
       <c r="H81" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K81" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="I81" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J81" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K81" s="2" t="s">
+      <c r="L81" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="L81" s="2" t="s">
-        <v>483</v>
-      </c>
       <c r="M81" s="2" t="s">
         <v>28</v>
       </c>
@@ -6806,18 +6795,18 @@
         <v>28</v>
       </c>
       <c r="S81" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="82" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>484</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>485</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>55</v>
@@ -6832,20 +6821,20 @@
         <v>25</v>
       </c>
       <c r="H82" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="I82" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K82" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="I82" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J82" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K82" s="2" t="s">
+      <c r="L82" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="L82" s="2" t="s">
-        <v>488</v>
-      </c>
       <c r="M82" s="2" t="s">
         <v>28</v>
       </c>
@@ -6865,18 +6854,18 @@
         <v>28</v>
       </c>
       <c r="S82" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="83" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>489</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>490</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>40</v>
@@ -6891,20 +6880,20 @@
         <v>25</v>
       </c>
       <c r="H83" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K83" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="I83" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J83" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K83" s="2" t="s">
+      <c r="L83" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="L83" s="2" t="s">
-        <v>493</v>
-      </c>
       <c r="M83" s="2" t="s">
         <v>28</v>
       </c>
@@ -6924,18 +6913,18 @@
         <v>28</v>
       </c>
       <c r="S83" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="84" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C84" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>495</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>55</v>
@@ -6950,20 +6939,20 @@
         <v>25</v>
       </c>
       <c r="H84" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K84" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="I84" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J84" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K84" s="2" t="s">
+      <c r="L84" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="L84" s="2" t="s">
-        <v>498</v>
-      </c>
       <c r="M84" s="2" t="s">
         <v>28</v>
       </c>
@@ -6983,18 +6972,18 @@
         <v>28</v>
       </c>
       <c r="S84" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="85" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>499</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>500</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>68</v>
@@ -7009,19 +6998,19 @@
         <v>25</v>
       </c>
       <c r="H85" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K85" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="I85" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J85" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K85" s="2" t="s">
+      <c r="L85" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="L85" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="M85" s="2" t="s">
         <v>28</v>
@@ -7039,21 +7028,21 @@
         <v>189</v>
       </c>
       <c r="R85" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="S85" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="86" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>505</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>506</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>68</v>
@@ -7068,19 +7057,19 @@
         <v>25</v>
       </c>
       <c r="H86" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="I86" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K86" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="I86" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="J86" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K86" s="2" t="s">
+      <c r="L86" s="2" t="s">
         <v>508</v>
-      </c>
-      <c r="L86" s="2" t="s">
-        <v>509</v>
       </c>
       <c r="M86" s="2" t="s">
         <v>28</v>
@@ -7098,10 +7087,10 @@
         <v>189</v>
       </c>
       <c r="R86" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="S86" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>